<commit_message>
Simplify prepared API-2008 conflict repair exercise
</commit_message>
<xml_diff>
--- a/test-cases.xlsx
+++ b/test-cases.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Summary" sheetId="1" r:id="Rababe841b4f9440f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="2" r:id="R1f7970dd6cce47e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Guide" sheetId="3" r:id="Raed39bbb3e9d4670"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Summary" sheetId="1" r:id="Raf396c4b995c4ee4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="2" r:id="R943b143b29aa4af1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Guide" sheetId="3" r:id="R8dd9b30be0fa4765"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -337,10 +337,10 @@
         <x:v>API-2008</x:v>
       </x:c>
       <x:c r="B2" s="4" t="str">
-        <x:v>A conflicting order preserves the active ride and succeeds after cancellation</x:v>
+        <x:v>A conflicting order preserves the active ride</x:v>
       </x:c>
       <x:c r="C2" s="4" t="str">
-        <x:v>Verify that a second ride request is rejected while a ride is active, leaves the original ride unchanged, and succeeds after that ride is cancelled.</x:v>
+        <x:v>Verify that a second ride request is rejected while a ride is active and leaves the original ride ID, route, tariff and status unchanged.</x:v>
       </x:c>
       <x:c r="D2" s="4" t="str">
         <x:v>A fresh authorized sandbox session exists with default settings and no active ride. Use the same bearer token and X-Sandbox-Session header for every request. Do not reset or replace the session between steps.</x:v>
@@ -349,18 +349,17 @@
         <x:v>regression, api, negative</x:v>
       </x:c>
       <x:c r="F2" s="4" t="str">
-        <x:v>api-tests/src/test/kotlin/tests/RideConflictRecoveryTest.kt#testConflictingOrderPreservesActiveRideAndAllowsRetryAfterCancellation</x:v>
+        <x:v>api-tests/src/test/kotlin/tests/RideConflictTest.kt#testConflictingOrderPreservesActiveRide</x:v>
       </x:c>
       <x:c r="G2" s="4" t="str">
         <x:v>POST /rides
-GET /rides/active
-POST /rides/{id}/cancel</x:v>
+GET /rides/active</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R977af933d3d7460f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea18e4b37a224ba4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -385,33 +384,25 @@
         <x:v>Expected Results</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="240" customHeight="1">
+    <x:row r="2" ht="135" customHeight="1">
       <x:c r="A2" s="4" t="str">
         <x:v>API-2008</x:v>
       </x:c>
       <x:c r="B2" s="4" t="str">
         <x:v>1. Send POST /rides with body {"from":"Oak Avenue","to":"Market Street","rideOptionId":1}. Retain the returned ride ID as rideAId.
 2. While ride A is active, send POST /rides with body {"from":"City Center","to":"Airport Terminal","rideOptionId":2}.
-3. Send GET /rides/active.
-4. Send POST /rides/{rideAId}/cancel using the ID retained in step 1.
-5. Send GET /rides/active.
-6. Repeat POST /rides with exactly the body from step 2. Retain the returned ride ID as rideBId.
-7. Send GET /rides/active.</x:v>
+3. Send GET /rides/active.</x:v>
       </x:c>
       <x:c r="C2" s="4" t="str">
         <x:v>1. HTTP 201. The ride has a positive ID, from "Oak Avenue", to "Market Street", option.id 1, and status "driver_found".
 2. HTTP 409. The error body contains error "An active ride already exists" and code "ACTIVE_RIDE_EXISTS".
-3. HTTP 200. The active ride still has id rideAId, from "Oak Avenue", to "Market Street", option.id 1, and status "driver_found".
-4. HTTP 200. The response has id rideAId and status "cancelled".
-5. HTTP 404. The error is "No active ride".
-6. HTTP 201. The ride has a positive ID different from rideAId, from "City Center", to "Airport Terminal", option.id 2, and status "driver_found".
-7. HTTP 200. The active ride has id rideBId, from "City Center", to "Airport Terminal", option.id 2, and status "driver_found".</x:v>
+3. HTTP 200. The active ride still has id rideAId, from "Oak Avenue", to "Market Street", option.id 1, and status "driver_found".</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5117e63856ec4825"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4908edf1a8a74d4b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>